<commit_message>
started working on t_test stuff and backing up old runs
</commit_message>
<xml_diff>
--- a/Results/Study 1/IoU_vals.xlsx
+++ b/Results/Study 1/IoU_vals.xlsx
@@ -682,10 +682,10 @@
         <v>3</v>
       </c>
       <c r="C2">
-        <v>0.2328219813559338</v>
+        <v>0.2663669908190274</v>
       </c>
       <c r="D2">
-        <v>0.3000851028237411</v>
+        <v>0.2959114886654339</v>
       </c>
     </row>
     <row r="3" spans="1:4">
@@ -696,10 +696,10 @@
         <v>4</v>
       </c>
       <c r="C3">
-        <v>0.2076756355433649</v>
+        <v>0.3505960588020458</v>
       </c>
       <c r="D3">
-        <v>0.2819984569956457</v>
+        <v>0.3865875081952964</v>
       </c>
     </row>
     <row r="4" spans="1:4">
@@ -710,10 +710,10 @@
         <v>5</v>
       </c>
       <c r="C4">
-        <v>0.2057856381073715</v>
+        <v>0.1807617542193758</v>
       </c>
       <c r="D4">
-        <v>0.3382783943122464</v>
+        <v>0.3649757378920139</v>
       </c>
     </row>
     <row r="5" spans="1:4">
@@ -724,10 +724,10 @@
         <v>6</v>
       </c>
       <c r="C5">
-        <v>0.07075304523613919</v>
+        <v>0.2359703628333926</v>
       </c>
       <c r="D5">
-        <v>0.2696785810111406</v>
+        <v>0.2023371376918493</v>
       </c>
     </row>
     <row r="6" spans="1:4">
@@ -738,10 +738,10 @@
         <v>7</v>
       </c>
       <c r="C6">
-        <v>0.2225858315168287</v>
+        <v>0.3016230518114372</v>
       </c>
       <c r="D6">
-        <v>0.3969616103328585</v>
+        <v>0.4214680710735317</v>
       </c>
     </row>
     <row r="7" spans="1:4">
@@ -752,10 +752,10 @@
         <v>8</v>
       </c>
       <c r="C7">
-        <v>0.1388434434967608</v>
+        <v>0.2142833640389742</v>
       </c>
       <c r="D7">
-        <v>0.3403296247432651</v>
+        <v>0.3313806233263226</v>
       </c>
     </row>
     <row r="8" spans="1:4">
@@ -766,10 +766,10 @@
         <v>9</v>
       </c>
       <c r="C8">
-        <v>0.2150534316631891</v>
+        <v>0.2856944748537261</v>
       </c>
       <c r="D8">
-        <v>0.3236561193592641</v>
+        <v>0.333351140575505</v>
       </c>
     </row>
     <row r="9" spans="1:4">
@@ -780,10 +780,10 @@
         <v>10</v>
       </c>
       <c r="C9">
-        <v>0.1300359175377629</v>
+        <v>0.2652413268612495</v>
       </c>
       <c r="D9">
-        <v>0.5569343748610376</v>
+        <v>0.3484872107367706</v>
       </c>
     </row>
     <row r="10" spans="1:4">
@@ -804,9 +804,6 @@
       <c r="B11" t="s">
         <v>12</v>
       </c>
-      <c r="D11">
-        <v>0.6588051279000614</v>
-      </c>
     </row>
     <row r="12" spans="1:4">
       <c r="A12" s="1">
@@ -815,6 +812,9 @@
       <c r="B12" t="s">
         <v>13</v>
       </c>
+      <c r="D12">
+        <v>0.5683010270220027</v>
+      </c>
     </row>
     <row r="13" spans="1:4">
       <c r="A13" s="1">
@@ -823,6 +823,9 @@
       <c r="B13" t="s">
         <v>14</v>
       </c>
+      <c r="D13">
+        <v>0.4519187551987157</v>
+      </c>
     </row>
     <row r="14" spans="1:4">
       <c r="A14" s="1">
@@ -832,7 +835,7 @@
         <v>15</v>
       </c>
       <c r="D14">
-        <v>0.5537513062003191</v>
+        <v>0.4645360975193972</v>
       </c>
     </row>
     <row r="15" spans="1:4">
@@ -850,9 +853,6 @@
       <c r="B16" t="s">
         <v>17</v>
       </c>
-      <c r="D16">
-        <v>0.5619995709192418</v>
-      </c>
     </row>
     <row r="17" spans="1:4">
       <c r="A17" s="1">
@@ -862,7 +862,7 @@
         <v>18</v>
       </c>
       <c r="D17">
-        <v>0.4978406192822236</v>
+        <v>0.5447464409814751</v>
       </c>
     </row>
   </sheetData>
@@ -902,10 +902,10 @@
         <v>4</v>
       </c>
       <c r="C3">
-        <v>0.2310940569902567</v>
+        <v>0.1898375787631454</v>
       </c>
       <c r="D3">
-        <v>0.2543080582342255</v>
+        <v>0.5263554302163123</v>
       </c>
     </row>
     <row r="4" spans="1:4">
@@ -915,12 +915,6 @@
       <c r="B4" t="s">
         <v>5</v>
       </c>
-      <c r="C4">
-        <v>0.2320966703211355</v>
-      </c>
-      <c r="D4">
-        <v>0.4277583216944068</v>
-      </c>
     </row>
     <row r="5" spans="1:4">
       <c r="A5" s="1">
@@ -930,10 +924,10 @@
         <v>6</v>
       </c>
       <c r="C5">
-        <v>0.1145664841887767</v>
+        <v>0.3400181722463242</v>
       </c>
       <c r="D5">
-        <v>0.3942415825648832</v>
+        <v>0.2340230629787181</v>
       </c>
     </row>
     <row r="6" spans="1:4">
@@ -952,10 +946,10 @@
         <v>8</v>
       </c>
       <c r="C7">
-        <v>0.2090282925184133</v>
+        <v>0.06323958904821775</v>
       </c>
       <c r="D7">
-        <v>0.2482817254648414</v>
+        <v>0.4307100465042158</v>
       </c>
     </row>
     <row r="8" spans="1:4">
@@ -965,12 +959,6 @@
       <c r="B8" t="s">
         <v>9</v>
       </c>
-      <c r="C8">
-        <v>0.1785319227421218</v>
-      </c>
-      <c r="D8">
-        <v>0.5519701157594633</v>
-      </c>
     </row>
     <row r="9" spans="1:4">
       <c r="A9" s="1">
@@ -980,10 +968,10 @@
         <v>10</v>
       </c>
       <c r="C9">
-        <v>0.1739770459877969</v>
+        <v>0.06694972010107422</v>
       </c>
       <c r="D9">
-        <v>0.5642376043701323</v>
+        <v>0.5639740800614312</v>
       </c>
     </row>
     <row r="10" spans="1:4">
@@ -1005,7 +993,7 @@
         <v>12</v>
       </c>
       <c r="D11">
-        <v>0.7200245464595698</v>
+        <v>0.5806333519397046</v>
       </c>
     </row>
     <row r="12" spans="1:4">
@@ -1016,7 +1004,7 @@
         <v>13</v>
       </c>
       <c r="D12">
-        <v>0.5869152567671183</v>
+        <v>0.55738367923766</v>
       </c>
     </row>
     <row r="13" spans="1:4">
@@ -1027,7 +1015,7 @@
         <v>14</v>
       </c>
       <c r="D13">
-        <v>0.339915086522682</v>
+        <v>0.5266833100559174</v>
       </c>
     </row>
     <row r="14" spans="1:4">
@@ -1038,7 +1026,7 @@
         <v>15</v>
       </c>
       <c r="D14">
-        <v>0.6788928091262262</v>
+        <v>0.4577535300667354</v>
       </c>
     </row>
     <row r="15" spans="1:4">
@@ -1049,7 +1037,7 @@
         <v>16</v>
       </c>
       <c r="D15">
-        <v>0.5836736618362609</v>
+        <v>0.6236622457326934</v>
       </c>
     </row>
     <row r="16" spans="1:4">
@@ -1060,7 +1048,7 @@
         <v>17</v>
       </c>
       <c r="D16">
-        <v>0.6209840934452766</v>
+        <v>0.6314377023158763</v>
       </c>
     </row>
     <row r="17" spans="1:4">
@@ -1071,7 +1059,7 @@
         <v>18</v>
       </c>
       <c r="D17">
-        <v>0.5552440308206211</v>
+        <v>0.532413617900356</v>
       </c>
     </row>
   </sheetData>
@@ -1103,10 +1091,10 @@
         <v>3</v>
       </c>
       <c r="C2">
-        <v>0.09291079261854868</v>
+        <v>0.04129751538079745</v>
       </c>
       <c r="D2">
-        <v>0.3619045409645429</v>
+        <v>0.5217447501611664</v>
       </c>
     </row>
     <row r="3" spans="1:4">
@@ -1117,10 +1105,10 @@
         <v>4</v>
       </c>
       <c r="C3">
-        <v>0.03285949905971491</v>
+        <v>0.08132735266292643</v>
       </c>
       <c r="D3">
-        <v>0.6316594876684046</v>
+        <v>0.4281625472945031</v>
       </c>
     </row>
     <row r="4" spans="1:4">
@@ -1131,10 +1119,10 @@
         <v>5</v>
       </c>
       <c r="C4">
-        <v>0.1846814470989338</v>
+        <v>0.09713029998670573</v>
       </c>
       <c r="D4">
-        <v>0.4603833131395064</v>
+        <v>0.5393066682534282</v>
       </c>
     </row>
     <row r="5" spans="1:4">
@@ -1145,10 +1133,10 @@
         <v>6</v>
       </c>
       <c r="C5">
-        <v>0.02219447038920956</v>
+        <v>0.03898045438694545</v>
       </c>
       <c r="D5">
-        <v>0.3633320711222356</v>
+        <v>0.4433400699883277</v>
       </c>
     </row>
     <row r="6" spans="1:4">
@@ -1159,10 +1147,10 @@
         <v>7</v>
       </c>
       <c r="C6">
-        <v>0.04741785527827119</v>
+        <v>0.2609282298530115</v>
       </c>
       <c r="D6">
-        <v>0.6222990213570541</v>
+        <v>0.4314480076463209</v>
       </c>
     </row>
     <row r="7" spans="1:4">
@@ -1173,10 +1161,10 @@
         <v>8</v>
       </c>
       <c r="C7">
-        <v>0.2088987803998869</v>
+        <v>0.007361044543885475</v>
       </c>
       <c r="D7">
-        <v>0.4749904376403722</v>
+        <v>0.5266076827999733</v>
       </c>
     </row>
     <row r="8" spans="1:4">
@@ -1187,10 +1175,10 @@
         <v>9</v>
       </c>
       <c r="C8">
-        <v>0.04713496181328528</v>
+        <v>0.1557065087638009</v>
       </c>
       <c r="D8">
-        <v>0.4183804707030549</v>
+        <v>0.6190528994767015</v>
       </c>
     </row>
     <row r="9" spans="1:4">
@@ -1201,10 +1189,10 @@
         <v>10</v>
       </c>
       <c r="C9">
-        <v>0.1792434705189005</v>
+        <v>0.3010764514532427</v>
       </c>
       <c r="D9">
-        <v>0.4418097399348662</v>
+        <v>0.5972285356236038</v>
       </c>
     </row>
     <row r="10" spans="1:4">
@@ -1226,7 +1214,7 @@
         <v>12</v>
       </c>
       <c r="D11">
-        <v>0.2401806662717356</v>
+        <v>0.4972693311138774</v>
       </c>
     </row>
     <row r="12" spans="1:4">
@@ -1237,7 +1225,7 @@
         <v>13</v>
       </c>
       <c r="D12">
-        <v>0.4164383885069346</v>
+        <v>0.3123970097631523</v>
       </c>
     </row>
     <row r="13" spans="1:4">
@@ -1248,7 +1236,7 @@
         <v>14</v>
       </c>
       <c r="D13">
-        <v>0.264017010468818</v>
+        <v>0.3322367411415351</v>
       </c>
     </row>
     <row r="14" spans="1:4">
@@ -1259,7 +1247,7 @@
         <v>15</v>
       </c>
       <c r="D14">
-        <v>0.4111736475109672</v>
+        <v>0.5093859481612624</v>
       </c>
     </row>
     <row r="15" spans="1:4">
@@ -1270,7 +1258,7 @@
         <v>16</v>
       </c>
       <c r="D15">
-        <v>0.4681678277957558</v>
+        <v>0.3300726194905237</v>
       </c>
     </row>
     <row r="16" spans="1:4">
@@ -1281,7 +1269,7 @@
         <v>17</v>
       </c>
       <c r="D16">
-        <v>0.4609526919205544</v>
+        <v>0.3184503185066802</v>
       </c>
     </row>
     <row r="17" spans="1:4">
@@ -1292,7 +1280,7 @@
         <v>18</v>
       </c>
       <c r="D17">
-        <v>0.1413121604898107</v>
+        <v>0.3465437254094342</v>
       </c>
     </row>
   </sheetData>
@@ -2772,10 +2760,10 @@
         <v>3</v>
       </c>
       <c r="C2">
-        <v>0.2574492853372347</v>
+        <v>0.2430938553879328</v>
       </c>
       <c r="D2">
-        <v>0.2233003643143899</v>
+        <v>0.1405330476909186</v>
       </c>
     </row>
     <row r="3" spans="1:4">
@@ -2786,10 +2774,10 @@
         <v>4</v>
       </c>
       <c r="C3">
-        <v>0.332257269590548</v>
+        <v>0.2670306376894491</v>
       </c>
       <c r="D3">
-        <v>0.2516343390403252</v>
+        <v>0.3230533027749524</v>
       </c>
     </row>
     <row r="4" spans="1:4">
@@ -2800,10 +2788,10 @@
         <v>5</v>
       </c>
       <c r="C4">
-        <v>0.2072104522947077</v>
+        <v>0.2582692647244548</v>
       </c>
       <c r="D4">
-        <v>0.2805586358058423</v>
+        <v>0.2927454807270018</v>
       </c>
     </row>
     <row r="5" spans="1:4">
@@ -2814,10 +2802,10 @@
         <v>6</v>
       </c>
       <c r="C5">
-        <v>0.2279982304943418</v>
+        <v>0.1685849217901815</v>
       </c>
       <c r="D5">
-        <v>0.1823768217669244</v>
+        <v>0.1502226568867375</v>
       </c>
     </row>
     <row r="6" spans="1:4">
@@ -2828,10 +2816,10 @@
         <v>7</v>
       </c>
       <c r="C6">
-        <v>0.2000472672146033</v>
+        <v>0.2368101516866529</v>
       </c>
       <c r="D6">
-        <v>0.3443025210543506</v>
+        <v>0.3482324010624037</v>
       </c>
     </row>
     <row r="7" spans="1:4">
@@ -2842,10 +2830,10 @@
         <v>8</v>
       </c>
       <c r="C7">
-        <v>0.1971351115861801</v>
+        <v>0.1665591368038207</v>
       </c>
       <c r="D7">
-        <v>0.2778158056123677</v>
+        <v>0.2893715948253022</v>
       </c>
     </row>
     <row r="8" spans="1:4">
@@ -2856,10 +2844,10 @@
         <v>9</v>
       </c>
       <c r="C8">
-        <v>0.2556358929403495</v>
+        <v>0.1821574918365189</v>
       </c>
       <c r="D8">
-        <v>0.2590564026075998</v>
+        <v>0.2837531582395693</v>
       </c>
     </row>
     <row r="9" spans="1:4">
@@ -2870,10 +2858,10 @@
         <v>10</v>
       </c>
       <c r="C9">
-        <v>0.2503734043915116</v>
+        <v>0.231893223686302</v>
       </c>
       <c r="D9">
-        <v>0.3467258830726783</v>
+        <v>0.3141561982692709</v>
       </c>
     </row>
     <row r="10" spans="1:4">
@@ -2895,7 +2883,7 @@
         <v>12</v>
       </c>
       <c r="D11">
-        <v>0.976565874567188</v>
+        <v>0.9735906667870986</v>
       </c>
     </row>
     <row r="12" spans="1:4">
@@ -2906,7 +2894,7 @@
         <v>13</v>
       </c>
       <c r="D12">
-        <v>0.9488137639749977</v>
+        <v>0.8939097603684802</v>
       </c>
     </row>
     <row r="13" spans="1:4">
@@ -2917,7 +2905,7 @@
         <v>14</v>
       </c>
       <c r="D13">
-        <v>0.8466233761651893</v>
+        <v>0.8988344310482842</v>
       </c>
     </row>
     <row r="14" spans="1:4">
@@ -2928,7 +2916,7 @@
         <v>15</v>
       </c>
       <c r="D14">
-        <v>0.9650644911183356</v>
+        <v>0.8458990452061064</v>
       </c>
     </row>
     <row r="15" spans="1:4">
@@ -2939,7 +2927,7 @@
         <v>16</v>
       </c>
       <c r="D15">
-        <v>0.9770205928073611</v>
+        <v>0.9493444051398897</v>
       </c>
     </row>
     <row r="16" spans="1:4">
@@ -2950,7 +2938,7 @@
         <v>17</v>
       </c>
       <c r="D16">
-        <v>0.9125624702001458</v>
+        <v>0.8744051806245413</v>
       </c>
     </row>
     <row r="17" spans="1:4">
@@ -2961,7 +2949,7 @@
         <v>18</v>
       </c>
       <c r="D17">
-        <v>0.9293871876223152</v>
+        <v>0.853200187283323</v>
       </c>
     </row>
   </sheetData>

</xml_diff>